<commit_message>
đang fix bug địa chỉ không khớp
</commit_message>
<xml_diff>
--- a/reports/trip_summary.xlsx
+++ b/reports/trip_summary.xlsx
@@ -529,19 +529,23 @@
       <c r="D2" t="n">
         <v>408.26</v>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>519.79</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.785</v>
+      </c>
       <c r="G2" t="n">
-        <v>315</v>
+        <v>239</v>
       </c>
       <c r="H2" t="b">
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -553,12 +557,14 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
+        <v>24.1</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="inlineStr"/>
+        <v>127172.8</v>
+      </c>
+      <c r="P2" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix origin set cứng
bổ sung phương thức tính toán cung đường không bắt buộc đếm đi và về phải trùng
</commit_message>
<xml_diff>
--- a/reports/trip_summary.xlsx
+++ b/reports/trip_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,396 +454,28 @@
           <t>Km kỳ vọng</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Tỷ lệ vòng</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Lệch tuyến</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Có quay đầu</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Điểm giao đã ghé</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Điểm giao bỏ sót</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Quay đầu hợp lệ</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Quay đầu nghi vấn</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Số vé ePass</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Tuân thủ hành lang (%)</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Lệch tối đa (m)</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Chân hàng tệ nhất</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>15068</t>
+          <t>14278</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>08:58</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>13:35</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>200.68</v>
+        <v>101.64</v>
       </c>
       <c r="E2" t="n">
-        <v>39.41</v>
-      </c>
-      <c r="F2" t="n">
-        <v>5.093</v>
-      </c>
-      <c r="G2" t="n">
-        <v>300</v>
-      </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L2" t="n">
-        <v>44</v>
-      </c>
-      <c r="M2" t="n">
-        <v>4</v>
-      </c>
-      <c r="N2" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="O2" t="n">
-        <v>30865.5</v>
-      </c>
-      <c r="P2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>18332</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>06:21</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>19:26</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>320.53</v>
-      </c>
-      <c r="E3" t="n">
-        <v>280.11</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1.144</v>
-      </c>
-      <c r="G3" t="n">
-        <v>169</v>
-      </c>
-      <c r="H3" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>14</v>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>5</v>
-      </c>
-      <c r="L3" t="n">
-        <v>8</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>46.3</v>
-      </c>
-      <c r="O3" t="n">
-        <v>18308.8</v>
-      </c>
-      <c r="P3" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>19142</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>03:51</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>18:27</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>303.84</v>
-      </c>
-      <c r="E4" t="n">
-        <v>251.02</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="G4" t="n">
-        <v>293</v>
-      </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>8</v>
-      </c>
-      <c r="J4" t="n">
-        <v>6</v>
-      </c>
-      <c r="K4" t="n">
-        <v>9</v>
-      </c>
-      <c r="L4" t="n">
-        <v>15</v>
-      </c>
-      <c r="M4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N4" t="n">
-        <v>7</v>
-      </c>
-      <c r="O4" t="n">
-        <v>52054.3</v>
-      </c>
-      <c r="P4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>19132</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>04:50</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>18:27</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>302.43</v>
-      </c>
-      <c r="E5" t="n">
-        <v>311.97</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="G5" t="n">
-        <v>223</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>13</v>
-      </c>
-      <c r="J5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>17</v>
-      </c>
-      <c r="M5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>29.2</v>
-      </c>
-      <c r="O5" t="n">
-        <v>63362.2</v>
-      </c>
-      <c r="P5" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>18856</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>04:44</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>18:02</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>258.12</v>
-      </c>
-      <c r="E6" t="n">
-        <v>212.04</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1.217</v>
-      </c>
-      <c r="G6" t="n">
-        <v>227</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>10</v>
-      </c>
-      <c r="J6" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" t="n">
-        <v>11</v>
-      </c>
-      <c r="L6" t="n">
-        <v>20</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="O6" t="n">
-        <v>42971.4</v>
-      </c>
-      <c r="P6" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>14278</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>08:58</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>14:56</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>101.64</v>
-      </c>
-      <c r="E7" t="n">
-        <v>66.20999999999999</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.535</v>
-      </c>
-      <c r="G7" t="n">
-        <v>148</v>
-      </c>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>9</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" t="n">
-        <v>7</v>
-      </c>
-      <c r="L7" t="n">
-        <v>16</v>
-      </c>
-      <c r="M7" t="n">
-        <v>2</v>
-      </c>
-      <c r="N7" t="n">
-        <v>53</v>
-      </c>
-      <c r="O7" t="n">
-        <v>6441.9</v>
-      </c>
-      <c r="P7" t="n">
-        <v>1</v>
+        <v>53.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>